<commit_message>
feat: add code for experimentation
</commit_message>
<xml_diff>
--- a/experimentacion_alpha.xlsx
+++ b/experimentacion_alpha.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="21">
   <si>
     <t xml:space="preserve">INITIAL_TEMPERATURE=1000 COOLING_RATE=0.95 MAX_ITERATIONS=1000000 COOLING_INTERVAL=50 MAX_STAGNATION=5000 SEED=42</t>
   </si>
@@ -31,6 +31,9 @@
     <t xml:space="preserve">(25) C101</t>
   </si>
   <si>
+    <t xml:space="preserve">SEED=42</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALPHA</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">(100) C101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEED=24</t>
   </si>
   <si>
     <t xml:space="preserve">(400) c1_4_1</t>
@@ -158,7 +164,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -168,6 +174,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -302,7 +312,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:F95"/>
+  <dimension ref="B2:G95"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.88"/>
@@ -323,22 +333,25 @@
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D4" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -357,6 +370,7 @@
       <c r="F7" s="2" t="n">
         <v>141.039</v>
       </c>
+      <c r="G7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="1" t="n">
@@ -482,24 +496,27 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -507,16 +524,16 @@
         <v>0</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>1275.96</v>
+        <v>1226.69</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>58253</v>
+        <v>57885.9</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>1275.96</v>
+        <v>1226.69</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -524,16 +541,16 @@
         <v>0.25</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>1361.71</v>
+        <v>1540.01</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>48.8076</v>
+        <v>0</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>1349.51</v>
+        <v>1540.01</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -541,16 +558,16 @@
         <v>0.5</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>1475.87</v>
+        <v>1817.22</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>0</v>
+        <v>3.45906</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>1475.87</v>
+        <v>1815.49</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -558,16 +575,16 @@
         <v>0.75</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>1481.79</v>
+        <v>1447.02</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>2.8304</v>
+        <v>0</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>1479.66</v>
+        <v>1447.02</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -575,7 +592,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>1766.31</v>
+        <v>1292.84</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>0</v>
@@ -584,7 +601,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>1766.31</v>
+        <v>1292.84</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -592,7 +609,7 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>1509.18</v>
+        <v>1332.85</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>0</v>
@@ -601,7 +618,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>1509.18</v>
+        <v>1332.85</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -609,7 +626,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>1715.88</v>
+        <v>1489.56</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>0</v>
@@ -618,7 +635,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>1715.88</v>
+        <v>1489.56</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -626,16 +643,16 @@
         <v>10</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>1763.81</v>
+        <v>1344.23</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="1" t="n">
-        <v>0</v>
+        <v>0.80464</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>1763.81</v>
+        <v>1336.18</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -643,24 +660,24 @@
         <v>1</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -804,24 +821,24 @@
         <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -965,30 +982,30 @@
         <v>1</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1081,30 +1098,30 @@
         <v>1</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1125,7 +1142,7 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="3" t="n">
+      <c r="B69" s="4" t="n">
         <v>0.97</v>
       </c>
       <c r="C69" s="1" t="n">
@@ -1142,7 +1159,7 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="3" t="n">
+      <c r="B70" s="4" t="n">
         <v>0.98</v>
       </c>
       <c r="C70" s="1" t="n">
@@ -1159,7 +1176,7 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="3" t="n">
+      <c r="B71" s="4" t="n">
         <v>0.99</v>
       </c>
       <c r="C71" s="1" t="n">
@@ -1176,7 +1193,7 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="3" t="n">
+      <c r="B72" s="4" t="n">
         <v>0.995</v>
       </c>
       <c r="C72" s="1" t="n">
@@ -1197,30 +1214,30 @@
         <v>1</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1344,27 +1361,27 @@
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1380,7 +1397,7 @@
       <c r="E89" s="1" t="n">
         <v>26412.4</v>
       </c>
-      <c r="F89" s="4" t="n">
+      <c r="F89" s="5" t="n">
         <v>424.399</v>
       </c>
     </row>

</xml_diff>